<commit_message>
Update generate_report.py and refresh extracted output files
- generate_report.py: 요약 시트 진행상태 행 추가, 건수/비율 한 줄 표시
- output/extracted, output/upload, output/reports: batch_run 최신 결과 반영
- data/existing: GT 파일 최신화

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/existing/판매중_상품구성_사업방법서_매핑.xlsx
+++ b/data/existing/판매중_상품구성_사업방법서_매핑.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\회사\문서자동화\사전자료\기준정보_260308\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\claudecsw\ruleautomatker\data\existing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14AB9043-5EF7-4832-B167-E5ABF933AEEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B446EF73-745F-4799-BCEC-BE4908B534A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{364CA86F-2012-40A9-A884-5853FC3C1200}"/>
+    <workbookView xWindow="51480" yWindow="30" windowWidth="51840" windowHeight="21120" xr2:uid="{364CA86F-2012-40A9-A884-5853FC3C1200}"/>
   </bookViews>
   <sheets>
     <sheet name="보종코드_상품코드_매핑" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">보종코드_상품코드_매핑!$A$1:$H$262</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">보종코드_상품코드_매핑!$A$1:$I$262</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1053" uniqueCount="455">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1054" uniqueCount="457">
   <si>
     <t>ISRN_KIND_DTCD</t>
   </si>
@@ -1275,133 +1275,142 @@
     <t>한화생명 H종신보험 무배당_사업방법서_20260101~.pdf</t>
   </si>
   <si>
+    <t>한화생명 Wealth단체저축보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 Wealth직장인연금보험 무배당_사업방법서_20260130~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 간편가입 H당뇨보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 간편가입 H종신보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 간편가입 Need AI 암보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 간편가입 경영인H정기보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 간편가입 상속H종신보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 간편가입 시그니처H보장보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 간편가입 시그니처H암보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 간편가입 실손의료비보장보험(갱신형) 무배당(재가입용)_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 간편가입 제로백H종신보험 무배당_사업방법서_20260201~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 간편가입 포켓골절보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 간편가입 하나로H종신보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 경영인H정기보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 기본형 급여 e실손의료비보장보험(갱신형) 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 기본형 급여 실손의료비보장보험(갱신형) 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 기본형 급여 실손의료비보장보험(계약전환 단체개인전환 개인중지재개용)(갱신형) 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 기업복지라이프플랜보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 노후실손의료비보장보험(갱신형) 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 바로연금보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 상생친구 보장보험 무배당_사업방법서_20260201~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 상속H종신보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 스마트H상해보험 무배당_사업방법서_20260201~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 스마트V상해보험 무배당_사업방법서_20260201~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 스마트V연금보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 스마트하이브리드연금보험 무배당_사업방법서_20260201~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 시그니처 H통합건강보험 무배당(납입면제형)_사업방법서_20260201~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 시그니처 H통합건강보험 무배당_사업방법서_20260201~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 시그니처H보장보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 시그니처H암보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 연금보험Enterprise 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 연금저축 미래로기업복지연금보험_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 연금저축 스마트하이드림연금보험_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 연금저축 하이드림연금보험_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 장애인전용 곰두리보장보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 제로백H종신보험 무배당_사업방법서_20260201~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 진심가득H보장보험 무배당_사업방법서_20260201~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 케어백간병플러스보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 튼튼이 치아보험(갱신형) 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 포켓골절보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>한화생명 하나로H종신보험 무배당_사업방법서_20260101~.pdf</t>
+  </si>
+  <si>
+    <t>사업방법서 파일명</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>한화생명 상속H종신보험 무배당_사업방법서_20260101~.pdf</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>한화생명 Need AI 암보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 Wealth단체저축보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 Wealth직장인연금보험 무배당_사업방법서_20260130~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 간편가입 H당뇨보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 간편가입 H종신보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 간편가입 Need AI 암보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 간편가입 경영인H정기보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 간편가입 상속H종신보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 간편가입 시그니처H보장보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 간편가입 시그니처H암보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 간편가입 실손의료비보장보험(갱신형) 무배당(재가입용)_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 간편가입 제로백H종신보험 무배당_사업방법서_20260201~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 간편가입 포켓골절보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 간편가입 하나로H종신보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 경영인H정기보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 기본형 급여 e실손의료비보장보험(갱신형) 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 기본형 급여 실손의료비보장보험(갱신형) 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 기본형 급여 실손의료비보장보험(계약전환 단체개인전환 개인중지재개용)(갱신형) 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 기업복지라이프플랜보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 노후실손의료비보장보험(갱신형) 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 바로연금보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 상생친구 보장보험 무배당_사업방법서_20260201~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 상속H종신보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 스마트H상해보험 무배당_사업방법서_20260201~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 스마트V상해보험 무배당_사업방법서_20260201~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 스마트V연금보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 스마트하이브리드연금보험 무배당_사업방법서_20260201~.pdf</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>한화생명 시그니처 H통합건강보험 무배당(납입면제형)_사업방법서_20260201~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 시그니처 H통합건강보험 무배당_사업방법서_20260201~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 시그니처H보장보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 시그니처H암보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 연금보험Enterprise 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 연금저축 미래로기업복지연금보험_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 연금저축 스마트하이드림연금보험_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 연금저축 하이드림연금보험_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 장애인전용 곰두리보장보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 제로백H종신보험 무배당_사업방법서_20260201~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 진심가득H보장보험 무배당_사업방법서_20260201~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 케어백간병플러스보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 튼튼이 치아보험(갱신형) 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 포켓골절보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>한화생명 하나로H종신보험 무배당_사업방법서_20260101~.pdf</t>
-  </si>
-  <si>
-    <t>사업방법서 파일명</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1775,7 +1784,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AECB136-8215-429B-82E5-8A6B6A669FFB}">
-  <dimension ref="A1:I262"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:N262"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.125" bestFit="1" customWidth="1"/>
@@ -1786,7 +1796,8 @@
     <col min="6" max="6" width="100.375" customWidth="1"/>
     <col min="7" max="7" width="24" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="23.875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="42" customWidth="1"/>
+    <col min="9" max="9" width="59.5" customWidth="1"/>
+    <col min="14" max="14" width="23.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
@@ -1815,10 +1826,10 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>454</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2061</v>
       </c>
@@ -1847,7 +1858,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2061</v>
       </c>
@@ -1876,7 +1887,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1772</v>
       </c>
@@ -1905,7 +1916,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1772</v>
       </c>
@@ -1934,7 +1945,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>1772</v>
       </c>
@@ -1963,7 +1974,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1772</v>
       </c>
@@ -1992,7 +2003,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1726</v>
       </c>
@@ -2021,7 +2032,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1726</v>
       </c>
@@ -2050,7 +2061,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>1726</v>
       </c>
@@ -2079,7 +2090,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>1726</v>
       </c>
@@ -2108,7 +2119,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>1764</v>
       </c>
@@ -2137,7 +2148,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>1764</v>
       </c>
@@ -2166,7 +2177,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>1764</v>
       </c>
@@ -2195,7 +2206,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>1764</v>
       </c>
@@ -2224,7 +2235,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2170</v>
       </c>
@@ -2253,7 +2264,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2170</v>
       </c>
@@ -2282,7 +2293,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>2170</v>
       </c>
@@ -2311,7 +2322,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>2246</v>
       </c>
@@ -2340,7 +2351,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2246</v>
       </c>
@@ -2369,7 +2380,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>2246</v>
       </c>
@@ -2398,7 +2409,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>2246</v>
       </c>
@@ -2427,7 +2438,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>2246</v>
       </c>
@@ -2456,7 +2467,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>2246</v>
       </c>
@@ -2485,7 +2496,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>2246</v>
       </c>
@@ -2514,7 +2525,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>2246</v>
       </c>
@@ -2543,7 +2554,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>2246</v>
       </c>
@@ -2572,7 +2583,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>2253</v>
       </c>
@@ -2601,7 +2612,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>2170</v>
       </c>
@@ -2630,7 +2641,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>2170</v>
       </c>
@@ -2659,7 +2670,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>2209</v>
       </c>
@@ -2688,7 +2699,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>2209</v>
       </c>
@@ -2717,7 +2728,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>2209</v>
       </c>
@@ -2746,7 +2757,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>2209</v>
       </c>
@@ -2775,7 +2786,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>2209</v>
       </c>
@@ -2804,7 +2815,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>2209</v>
       </c>
@@ -2833,7 +2844,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>2209</v>
       </c>
@@ -2862,7 +2873,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>2209</v>
       </c>
@@ -2891,7 +2902,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>2248</v>
       </c>
@@ -2917,10 +2928,10 @@
         <v>2958465</v>
       </c>
       <c r="I39" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>1796</v>
       </c>
@@ -2946,10 +2957,10 @@
         <v>2958465</v>
       </c>
       <c r="I40" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>1833</v>
       </c>
@@ -2975,10 +2986,10 @@
         <v>2958465</v>
       </c>
       <c r="I41" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>1833</v>
       </c>
@@ -3004,10 +3015,10 @@
         <v>2958465</v>
       </c>
       <c r="I42" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>2254</v>
       </c>
@@ -3033,10 +3044,10 @@
         <v>2958465</v>
       </c>
       <c r="I43" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>2210</v>
       </c>
@@ -3062,10 +3073,10 @@
         <v>2958465</v>
       </c>
       <c r="I44" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>2210</v>
       </c>
@@ -3091,10 +3102,10 @@
         <v>2958465</v>
       </c>
       <c r="I45" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>2210</v>
       </c>
@@ -3120,10 +3131,10 @@
         <v>2958465</v>
       </c>
       <c r="I46" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>2210</v>
       </c>
@@ -3149,10 +3160,10 @@
         <v>2958465</v>
       </c>
       <c r="I47" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>2249</v>
       </c>
@@ -3178,10 +3189,10 @@
         <v>2958465</v>
       </c>
       <c r="I48" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>2249</v>
       </c>
@@ -3207,10 +3218,10 @@
         <v>2958465</v>
       </c>
       <c r="I49" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>2243</v>
       </c>
@@ -3236,10 +3247,10 @@
         <v>2958465</v>
       </c>
       <c r="I50" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>2243</v>
       </c>
@@ -3265,10 +3276,10 @@
         <v>2958465</v>
       </c>
       <c r="I51" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>2130</v>
       </c>
@@ -3294,10 +3305,10 @@
         <v>2958465</v>
       </c>
       <c r="I52" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>2130</v>
       </c>
@@ -3323,10 +3334,10 @@
         <v>2958465</v>
       </c>
       <c r="I53" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>2205</v>
       </c>
@@ -3352,10 +3363,10 @@
         <v>2958465</v>
       </c>
       <c r="I54" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>2205</v>
       </c>
@@ -3381,10 +3392,10 @@
         <v>2958465</v>
       </c>
       <c r="I55" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>1976</v>
       </c>
@@ -3410,10 +3421,10 @@
         <v>2958465</v>
       </c>
       <c r="I56" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>1976</v>
       </c>
@@ -3439,10 +3450,10 @@
         <v>2958465</v>
       </c>
       <c r="I57" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>1976</v>
       </c>
@@ -3468,10 +3479,10 @@
         <v>2958465</v>
       </c>
       <c r="I58" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>1976</v>
       </c>
@@ -3497,10 +3508,10 @@
         <v>2958465</v>
       </c>
       <c r="I59" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>2208</v>
       </c>
@@ -3526,10 +3537,10 @@
         <v>2958465</v>
       </c>
       <c r="I60" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>2208</v>
       </c>
@@ -3555,10 +3566,10 @@
         <v>2958465</v>
       </c>
       <c r="I61" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>2256</v>
       </c>
@@ -3584,10 +3595,10 @@
         <v>2958465</v>
       </c>
       <c r="I62" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>2251</v>
       </c>
@@ -3613,10 +3624,10 @@
         <v>2958465</v>
       </c>
       <c r="I63" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>2251</v>
       </c>
@@ -3642,10 +3653,10 @@
         <v>2958465</v>
       </c>
       <c r="I64" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>2251</v>
       </c>
@@ -3671,10 +3682,10 @@
         <v>2958465</v>
       </c>
       <c r="I65" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>2242</v>
       </c>
@@ -3700,10 +3711,10 @@
         <v>2958465</v>
       </c>
       <c r="I66" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>2242</v>
       </c>
@@ -3729,10 +3740,10 @@
         <v>2958465</v>
       </c>
       <c r="I67" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>2242</v>
       </c>
@@ -3758,10 +3769,10 @@
         <v>2958465</v>
       </c>
       <c r="I68" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>2242</v>
       </c>
@@ -3787,10 +3798,10 @@
         <v>2958465</v>
       </c>
       <c r="I69" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>1983</v>
       </c>
@@ -3816,10 +3827,10 @@
         <v>2958465</v>
       </c>
       <c r="I70" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>1983</v>
       </c>
@@ -3845,10 +3856,10 @@
         <v>2958465</v>
       </c>
       <c r="I71" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>1982</v>
       </c>
@@ -3874,10 +3885,10 @@
         <v>2958465</v>
       </c>
       <c r="I72" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>1982</v>
       </c>
@@ -3903,10 +3914,10 @@
         <v>2958465</v>
       </c>
       <c r="I73" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>1982</v>
       </c>
@@ -3932,10 +3943,10 @@
         <v>2958465</v>
       </c>
       <c r="I74" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>1982</v>
       </c>
@@ -3961,10 +3972,10 @@
         <v>2958465</v>
       </c>
       <c r="I75" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>1984</v>
       </c>
@@ -3990,10 +4001,10 @@
         <v>2958465</v>
       </c>
       <c r="I76" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>1984</v>
       </c>
@@ -4019,10 +4030,10 @@
         <v>2958465</v>
       </c>
       <c r="I77" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>1984</v>
       </c>
@@ -4048,10 +4059,10 @@
         <v>2958465</v>
       </c>
       <c r="I78" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>1984</v>
       </c>
@@ -4077,10 +4088,10 @@
         <v>2958465</v>
       </c>
       <c r="I79" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>1984</v>
       </c>
@@ -4106,10 +4117,10 @@
         <v>2958465</v>
       </c>
       <c r="I80" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.3">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>1984</v>
       </c>
@@ -4135,10 +4146,10 @@
         <v>2958465</v>
       </c>
       <c r="I81" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.3">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>1984</v>
       </c>
@@ -4164,10 +4175,10 @@
         <v>2958465</v>
       </c>
       <c r="I82" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>1984</v>
       </c>
@@ -4193,10 +4204,10 @@
         <v>2958465</v>
       </c>
       <c r="I83" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>1985</v>
       </c>
@@ -4222,10 +4233,10 @@
         <v>2958465</v>
       </c>
       <c r="I84" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>1985</v>
       </c>
@@ -4251,10 +4262,10 @@
         <v>2958465</v>
       </c>
       <c r="I85" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>1985</v>
       </c>
@@ -4280,10 +4291,10 @@
         <v>2958465</v>
       </c>
       <c r="I86" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>1985</v>
       </c>
@@ -4309,10 +4320,10 @@
         <v>2958465</v>
       </c>
       <c r="I87" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>1986</v>
       </c>
@@ -4338,10 +4349,10 @@
         <v>2958465</v>
       </c>
       <c r="I88" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>1986</v>
       </c>
@@ -4367,10 +4378,10 @@
         <v>2958465</v>
       </c>
       <c r="I89" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>1224</v>
       </c>
@@ -4396,10 +4407,10 @@
         <v>2958465</v>
       </c>
       <c r="I90" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.3">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>1224</v>
       </c>
@@ -4425,10 +4436,10 @@
         <v>2958465</v>
       </c>
       <c r="I91" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>1808</v>
       </c>
@@ -4454,10 +4465,10 @@
         <v>2958465</v>
       </c>
       <c r="I92" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>1808</v>
       </c>
@@ -4483,10 +4494,10 @@
         <v>2958465</v>
       </c>
       <c r="I93" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>1946</v>
       </c>
@@ -4512,10 +4523,10 @@
         <v>2958465</v>
       </c>
       <c r="I94" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.3">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>1946</v>
       </c>
@@ -4541,10 +4552,10 @@
         <v>2958465</v>
       </c>
       <c r="I95" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.3">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>2259</v>
       </c>
@@ -4570,10 +4581,10 @@
         <v>2958465</v>
       </c>
       <c r="I96" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>2259</v>
       </c>
@@ -4599,10 +4610,10 @@
         <v>2958465</v>
       </c>
       <c r="I97" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>2259</v>
       </c>
@@ -4628,10 +4639,10 @@
         <v>2958465</v>
       </c>
       <c r="I98" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>2259</v>
       </c>
@@ -4657,10 +4668,10 @@
         <v>2958465</v>
       </c>
       <c r="I99" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>2259</v>
       </c>
@@ -4686,10 +4697,10 @@
         <v>2958465</v>
       </c>
       <c r="I100" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>2259</v>
       </c>
@@ -4715,10 +4726,10 @@
         <v>2958465</v>
       </c>
       <c r="I101" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>2259</v>
       </c>
@@ -4744,10 +4755,10 @@
         <v>2958465</v>
       </c>
       <c r="I102" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>2259</v>
       </c>
@@ -4773,10 +4784,10 @@
         <v>2958465</v>
       </c>
       <c r="I103" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>2259</v>
       </c>
@@ -4802,10 +4813,10 @@
         <v>2958465</v>
       </c>
       <c r="I104" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>2259</v>
       </c>
@@ -4831,10 +4842,10 @@
         <v>2958465</v>
       </c>
       <c r="I105" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>2259</v>
       </c>
@@ -4860,10 +4871,10 @@
         <v>2958465</v>
       </c>
       <c r="I106" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>2259</v>
       </c>
@@ -4889,10 +4900,10 @@
         <v>2958465</v>
       </c>
       <c r="I107" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>2259</v>
       </c>
@@ -4918,10 +4929,10 @@
         <v>2958465</v>
       </c>
       <c r="I108" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>2259</v>
       </c>
@@ -4947,10 +4958,10 @@
         <v>2958465</v>
       </c>
       <c r="I109" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>2259</v>
       </c>
@@ -4976,10 +4987,10 @@
         <v>2958465</v>
       </c>
       <c r="I110" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>2259</v>
       </c>
@@ -5005,10 +5016,10 @@
         <v>2958465</v>
       </c>
       <c r="I111" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>2259</v>
       </c>
@@ -5034,10 +5045,10 @@
         <v>2958465</v>
       </c>
       <c r="I112" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>2259</v>
       </c>
@@ -5063,10 +5074,10 @@
         <v>2958465</v>
       </c>
       <c r="I113" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>2259</v>
       </c>
@@ -5092,10 +5103,10 @@
         <v>2958465</v>
       </c>
       <c r="I114" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>2259</v>
       </c>
@@ -5121,10 +5132,10 @@
         <v>2958465</v>
       </c>
       <c r="I115" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>2259</v>
       </c>
@@ -5150,10 +5161,10 @@
         <v>2958465</v>
       </c>
       <c r="I116" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>2259</v>
       </c>
@@ -5179,10 +5190,10 @@
         <v>2958465</v>
       </c>
       <c r="I117" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>2126</v>
       </c>
@@ -5208,10 +5219,10 @@
         <v>2958465</v>
       </c>
       <c r="I118" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.3">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>2126</v>
       </c>
@@ -5237,10 +5248,10 @@
         <v>2958465</v>
       </c>
       <c r="I119" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.3">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>2126</v>
       </c>
@@ -5266,10 +5277,10 @@
         <v>2958465</v>
       </c>
       <c r="I120" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.3">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="121" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>2129</v>
       </c>
@@ -5295,10 +5306,10 @@
         <v>2958465</v>
       </c>
       <c r="I121" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.3">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="122" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>2129</v>
       </c>
@@ -5324,10 +5335,10 @@
         <v>2958465</v>
       </c>
       <c r="I122" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.3">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="123" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>2129</v>
       </c>
@@ -5353,10 +5364,10 @@
         <v>2958465</v>
       </c>
       <c r="I123" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.3">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>2129</v>
       </c>
@@ -5382,10 +5393,10 @@
         <v>2958465</v>
       </c>
       <c r="I124" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.3">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>2236</v>
       </c>
@@ -5411,10 +5422,10 @@
         <v>2958465</v>
       </c>
       <c r="I125" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.3">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="126" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>2236</v>
       </c>
@@ -5440,10 +5451,10 @@
         <v>2958465</v>
       </c>
       <c r="I126" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.3">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="127" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>2236</v>
       </c>
@@ -5469,10 +5480,10 @@
         <v>2958465</v>
       </c>
       <c r="I127" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.3">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="128" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>2236</v>
       </c>
@@ -5498,10 +5509,10 @@
         <v>2958465</v>
       </c>
       <c r="I128" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.3">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="129" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>1758</v>
       </c>
@@ -5527,10 +5538,10 @@
         <v>2958465</v>
       </c>
       <c r="I129" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="130" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>1758</v>
       </c>
@@ -5556,10 +5567,10 @@
         <v>2958465</v>
       </c>
       <c r="I130" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="131" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>1758</v>
       </c>
@@ -5585,10 +5596,10 @@
         <v>2958465</v>
       </c>
       <c r="I131" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="132" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>1758</v>
       </c>
@@ -5614,10 +5625,10 @@
         <v>2958465</v>
       </c>
       <c r="I132" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="133" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>1758</v>
       </c>
@@ -5643,10 +5654,10 @@
         <v>2958465</v>
       </c>
       <c r="I133" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="134" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>2042</v>
       </c>
@@ -5672,10 +5683,10 @@
         <v>2958465</v>
       </c>
       <c r="I134" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.3">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="135" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>2042</v>
       </c>
@@ -5701,10 +5712,10 @@
         <v>2958465</v>
       </c>
       <c r="I135" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.3">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="136" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>2042</v>
       </c>
@@ -5730,10 +5741,10 @@
         <v>2958465</v>
       </c>
       <c r="I136" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.3">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="137" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>2042</v>
       </c>
@@ -5759,10 +5770,10 @@
         <v>2958465</v>
       </c>
       <c r="I137" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.3">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="138" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>2042</v>
       </c>
@@ -5788,10 +5799,10 @@
         <v>2958465</v>
       </c>
       <c r="I138" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.3">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="139" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>2258</v>
       </c>
@@ -5817,10 +5828,10 @@
         <v>2958465</v>
       </c>
       <c r="I139" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.3">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="140" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>2258</v>
       </c>
@@ -5846,10 +5857,17 @@
         <v>2958465</v>
       </c>
       <c r="I140" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.3">
+        <v>438</v>
+      </c>
+      <c r="M140">
+        <f>IF(I139=N140,1,2)</f>
+        <v>1</v>
+      </c>
+      <c r="N140" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="141" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>2258</v>
       </c>
@@ -5875,10 +5893,10 @@
         <v>2958465</v>
       </c>
       <c r="I141" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.3">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="142" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>2258</v>
       </c>
@@ -5904,10 +5922,10 @@
         <v>2958465</v>
       </c>
       <c r="I142" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.3">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="143" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>2258</v>
       </c>
@@ -5933,10 +5951,10 @@
         <v>2958465</v>
       </c>
       <c r="I143" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.3">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="144" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>2258</v>
       </c>
@@ -5962,7 +5980,7 @@
         <v>2958465</v>
       </c>
       <c r="I144" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.3">
@@ -5991,7 +6009,7 @@
         <v>2958465</v>
       </c>
       <c r="I145" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.3">
@@ -6020,7 +6038,7 @@
         <v>2958465</v>
       </c>
       <c r="I146" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.3">
@@ -6049,7 +6067,7 @@
         <v>2958465</v>
       </c>
       <c r="I147" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.3">
@@ -6078,7 +6096,7 @@
         <v>2958465</v>
       </c>
       <c r="I148" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.3">
@@ -6107,7 +6125,7 @@
         <v>2958465</v>
       </c>
       <c r="I149" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.3">
@@ -6136,7 +6154,7 @@
         <v>2958465</v>
       </c>
       <c r="I150" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.3">
@@ -6165,10 +6183,10 @@
         <v>2958465</v>
       </c>
       <c r="I151" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.3">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="152" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>2257</v>
       </c>
@@ -6194,10 +6212,10 @@
         <v>2958465</v>
       </c>
       <c r="I152" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.3">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="153" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>2257</v>
       </c>
@@ -6223,10 +6241,10 @@
         <v>2958465</v>
       </c>
       <c r="I153" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.3">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>2257</v>
       </c>
@@ -6252,10 +6270,10 @@
         <v>2958465</v>
       </c>
       <c r="I154" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.3">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="155" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>2257</v>
       </c>
@@ -6281,10 +6299,10 @@
         <v>2958465</v>
       </c>
       <c r="I155" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.3">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="156" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>2257</v>
       </c>
@@ -6310,10 +6328,10 @@
         <v>2958465</v>
       </c>
       <c r="I156" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.3">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="157" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>2257</v>
       </c>
@@ -6339,10 +6357,10 @@
         <v>2958465</v>
       </c>
       <c r="I157" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.3">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="158" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>2257</v>
       </c>
@@ -6368,10 +6386,10 @@
         <v>2958465</v>
       </c>
       <c r="I158" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.3">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="159" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>2257</v>
       </c>
@@ -6397,10 +6415,10 @@
         <v>2958465</v>
       </c>
       <c r="I159" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.3">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="160" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>2257</v>
       </c>
@@ -6426,10 +6444,10 @@
         <v>2958465</v>
       </c>
       <c r="I160" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.3">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="161" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>2257</v>
       </c>
@@ -6455,10 +6473,10 @@
         <v>2958465</v>
       </c>
       <c r="I161" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.3">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="162" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>2257</v>
       </c>
@@ -6484,10 +6502,10 @@
         <v>2958465</v>
       </c>
       <c r="I162" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="163" spans="1:9" x14ac:dyDescent="0.3">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="163" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>2257</v>
       </c>
@@ -6513,10 +6531,10 @@
         <v>2958465</v>
       </c>
       <c r="I163" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.3">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="164" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>2257</v>
       </c>
@@ -6542,10 +6560,10 @@
         <v>2958465</v>
       </c>
       <c r="I164" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="165" spans="1:9" x14ac:dyDescent="0.3">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="165" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>2204</v>
       </c>
@@ -6571,10 +6589,10 @@
         <v>2958465</v>
       </c>
       <c r="I165" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="166" spans="1:9" x14ac:dyDescent="0.3">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="166" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>2204</v>
       </c>
@@ -6600,10 +6618,10 @@
         <v>2958465</v>
       </c>
       <c r="I166" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.3">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="167" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>1571</v>
       </c>
@@ -6629,10 +6647,10 @@
         <v>2958465</v>
       </c>
       <c r="I167" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="168" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="168" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>1571</v>
       </c>
@@ -6658,10 +6676,10 @@
         <v>2958465</v>
       </c>
       <c r="I168" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="169" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="169" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>1571</v>
       </c>
@@ -6687,10 +6705,10 @@
         <v>2958465</v>
       </c>
       <c r="I169" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="170" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="170" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>1571</v>
       </c>
@@ -6716,10 +6734,10 @@
         <v>2958465</v>
       </c>
       <c r="I170" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="171" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>1571</v>
       </c>
@@ -6745,10 +6763,10 @@
         <v>2958465</v>
       </c>
       <c r="I171" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="172" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>1571</v>
       </c>
@@ -6774,10 +6792,10 @@
         <v>2958465</v>
       </c>
       <c r="I172" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="173" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>1571</v>
       </c>
@@ -6803,10 +6821,10 @@
         <v>2958465</v>
       </c>
       <c r="I173" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="174" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>1571</v>
       </c>
@@ -6832,10 +6850,10 @@
         <v>2958465</v>
       </c>
       <c r="I174" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="175" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>1571</v>
       </c>
@@ -6861,10 +6879,10 @@
         <v>2958465</v>
       </c>
       <c r="I175" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="176" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>1571</v>
       </c>
@@ -6890,10 +6908,10 @@
         <v>2958465</v>
       </c>
       <c r="I176" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="177" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="177" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>1571</v>
       </c>
@@ -6919,10 +6937,10 @@
         <v>2958465</v>
       </c>
       <c r="I177" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="178" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="178" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>1571</v>
       </c>
@@ -6948,10 +6966,10 @@
         <v>2958465</v>
       </c>
       <c r="I178" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="179" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="179" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>1571</v>
       </c>
@@ -6977,10 +6995,10 @@
         <v>2958465</v>
       </c>
       <c r="I179" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="180" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="180" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>1571</v>
       </c>
@@ -7006,10 +7024,10 @@
         <v>2958465</v>
       </c>
       <c r="I180" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="181" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="181" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>1571</v>
       </c>
@@ -7035,10 +7053,10 @@
         <v>2958465</v>
       </c>
       <c r="I181" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="182" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="182" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>1571</v>
       </c>
@@ -7064,10 +7082,10 @@
         <v>2958465</v>
       </c>
       <c r="I182" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="183" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="183" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>1571</v>
       </c>
@@ -7093,10 +7111,10 @@
         <v>2958465</v>
       </c>
       <c r="I183" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="184" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="184" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>1571</v>
       </c>
@@ -7122,10 +7140,10 @@
         <v>2958465</v>
       </c>
       <c r="I184" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="185" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="185" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>1571</v>
       </c>
@@ -7151,10 +7169,10 @@
         <v>2958465</v>
       </c>
       <c r="I185" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="186" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="186" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>1571</v>
       </c>
@@ -7180,10 +7198,10 @@
         <v>2958465</v>
       </c>
       <c r="I186" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="187" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="187" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>1571</v>
       </c>
@@ -7209,10 +7227,10 @@
         <v>2958465</v>
       </c>
       <c r="I187" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="188" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="188" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>1571</v>
       </c>
@@ -7238,10 +7256,10 @@
         <v>2958465</v>
       </c>
       <c r="I188" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="189" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="189" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>1571</v>
       </c>
@@ -7267,10 +7285,10 @@
         <v>2958465</v>
       </c>
       <c r="I189" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="190" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="190" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>1571</v>
       </c>
@@ -7296,10 +7314,10 @@
         <v>2958465</v>
       </c>
       <c r="I190" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="191" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="191" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>1571</v>
       </c>
@@ -7325,10 +7343,10 @@
         <v>2958465</v>
       </c>
       <c r="I191" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="192" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="192" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>1571</v>
       </c>
@@ -7354,10 +7372,10 @@
         <v>2958465</v>
       </c>
       <c r="I192" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="193" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="193" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>1571</v>
       </c>
@@ -7383,10 +7401,10 @@
         <v>2958465</v>
       </c>
       <c r="I193" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="194" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="194" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>1571</v>
       </c>
@@ -7412,10 +7430,10 @@
         <v>2958465</v>
       </c>
       <c r="I194" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="195" spans="1:9" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="195" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>1629</v>
       </c>
@@ -7441,10 +7459,10 @@
         <v>2958465</v>
       </c>
       <c r="I195" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="196" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="196" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>1629</v>
       </c>
@@ -7470,10 +7488,10 @@
         <v>2958465</v>
       </c>
       <c r="I196" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="197" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="197" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>1629</v>
       </c>
@@ -7499,10 +7517,10 @@
         <v>2958465</v>
       </c>
       <c r="I197" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="198" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="198" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>1629</v>
       </c>
@@ -7528,10 +7546,10 @@
         <v>2958465</v>
       </c>
       <c r="I198" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="199" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="199" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>1629</v>
       </c>
@@ -7557,10 +7575,10 @@
         <v>2958465</v>
       </c>
       <c r="I199" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="200" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="200" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>1629</v>
       </c>
@@ -7586,10 +7604,10 @@
         <v>2958465</v>
       </c>
       <c r="I200" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="201" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="201" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>1629</v>
       </c>
@@ -7615,10 +7633,10 @@
         <v>2958465</v>
       </c>
       <c r="I201" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="202" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="202" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>1809</v>
       </c>
@@ -7644,10 +7662,10 @@
         <v>2958465</v>
       </c>
       <c r="I202" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="203" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="203" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>1809</v>
       </c>
@@ -7673,10 +7691,10 @@
         <v>2958465</v>
       </c>
       <c r="I203" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="204" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="204" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>1809</v>
       </c>
@@ -7702,10 +7720,10 @@
         <v>2958465</v>
       </c>
       <c r="I204" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="205" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="205" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>1809</v>
       </c>
@@ -7731,10 +7749,10 @@
         <v>2958465</v>
       </c>
       <c r="I205" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="206" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="206" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>1809</v>
       </c>
@@ -7760,10 +7778,10 @@
         <v>2958465</v>
       </c>
       <c r="I206" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="207" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="207" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>1809</v>
       </c>
@@ -7789,10 +7807,10 @@
         <v>2958465</v>
       </c>
       <c r="I207" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="208" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="208" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>1809</v>
       </c>
@@ -7818,10 +7836,10 @@
         <v>2958465</v>
       </c>
       <c r="I208" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="209" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="209" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>1809</v>
       </c>
@@ -7847,10 +7865,10 @@
         <v>2958465</v>
       </c>
       <c r="I209" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="210" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="210" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>1809</v>
       </c>
@@ -7876,10 +7894,10 @@
         <v>2958465</v>
       </c>
       <c r="I210" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="211" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="211" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>1809</v>
       </c>
@@ -7905,10 +7923,10 @@
         <v>2958465</v>
       </c>
       <c r="I211" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="212" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="212" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>1809</v>
       </c>
@@ -7934,10 +7952,10 @@
         <v>2958465</v>
       </c>
       <c r="I212" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="213" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="213" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>1809</v>
       </c>
@@ -7963,10 +7981,10 @@
         <v>2958465</v>
       </c>
       <c r="I213" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="214" spans="1:9" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="214" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>1228</v>
       </c>
@@ -7992,10 +8010,10 @@
         <v>2958465</v>
       </c>
       <c r="I214" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="215" spans="1:9" x14ac:dyDescent="0.3">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="215" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>1228</v>
       </c>
@@ -8021,10 +8039,10 @@
         <v>2958465</v>
       </c>
       <c r="I215" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="216" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="216" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>1745</v>
       </c>
@@ -8050,10 +8068,10 @@
         <v>2958465</v>
       </c>
       <c r="I216" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="217" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="217" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>1745</v>
       </c>
@@ -8079,10 +8097,10 @@
         <v>2958465</v>
       </c>
       <c r="I217" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="218" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="218" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>1745</v>
       </c>
@@ -8108,10 +8126,10 @@
         <v>2958465</v>
       </c>
       <c r="I218" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="219" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="219" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>1745</v>
       </c>
@@ -8137,10 +8155,10 @@
         <v>2958465</v>
       </c>
       <c r="I219" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="220" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="220" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A220">
         <v>1745</v>
       </c>
@@ -8166,10 +8184,10 @@
         <v>2958465</v>
       </c>
       <c r="I220" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="221" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="221" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A221">
         <v>1745</v>
       </c>
@@ -8195,10 +8213,10 @@
         <v>2958465</v>
       </c>
       <c r="I221" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="222" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="222" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A222">
         <v>1745</v>
       </c>
@@ -8224,10 +8242,10 @@
         <v>2958465</v>
       </c>
       <c r="I222" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="223" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="223" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A223">
         <v>1745</v>
       </c>
@@ -8253,10 +8271,10 @@
         <v>2958465</v>
       </c>
       <c r="I223" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="224" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="224" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A224">
         <v>1745</v>
       </c>
@@ -8282,10 +8300,10 @@
         <v>2958465</v>
       </c>
       <c r="I224" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="225" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="225" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A225">
         <v>1745</v>
       </c>
@@ -8311,10 +8329,10 @@
         <v>2958465</v>
       </c>
       <c r="I225" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="226" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="226" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A226">
         <v>1745</v>
       </c>
@@ -8340,10 +8358,10 @@
         <v>2958465</v>
       </c>
       <c r="I226" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="227" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="227" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A227">
         <v>1745</v>
       </c>
@@ -8369,10 +8387,10 @@
         <v>2958465</v>
       </c>
       <c r="I227" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="228" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="228" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A228">
         <v>1745</v>
       </c>
@@ -8398,10 +8416,10 @@
         <v>2958465</v>
       </c>
       <c r="I228" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="229" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="229" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A229">
         <v>1745</v>
       </c>
@@ -8427,10 +8445,10 @@
         <v>2958465</v>
       </c>
       <c r="I229" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="230" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="230" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A230">
         <v>1745</v>
       </c>
@@ -8456,10 +8474,10 @@
         <v>2958465</v>
       </c>
       <c r="I230" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="231" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="231" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A231">
         <v>1745</v>
       </c>
@@ -8485,10 +8503,10 @@
         <v>2958465</v>
       </c>
       <c r="I231" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="232" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="232" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A232">
         <v>1745</v>
       </c>
@@ -8514,10 +8532,10 @@
         <v>2958465</v>
       </c>
       <c r="I232" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="233" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="233" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A233">
         <v>1745</v>
       </c>
@@ -8543,10 +8561,10 @@
         <v>2958465</v>
       </c>
       <c r="I233" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="234" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="234" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A234">
         <v>1745</v>
       </c>
@@ -8572,10 +8590,10 @@
         <v>2958465</v>
       </c>
       <c r="I234" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="235" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="235" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A235">
         <v>1745</v>
       </c>
@@ -8601,10 +8619,10 @@
         <v>2958465</v>
       </c>
       <c r="I235" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="236" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="236" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A236">
         <v>1745</v>
       </c>
@@ -8630,10 +8648,10 @@
         <v>2958465</v>
       </c>
       <c r="I236" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="237" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="237" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A237">
         <v>1745</v>
       </c>
@@ -8659,10 +8677,10 @@
         <v>2958465</v>
       </c>
       <c r="I237" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="238" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="238" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A238">
         <v>1745</v>
       </c>
@@ -8688,10 +8706,10 @@
         <v>2958465</v>
       </c>
       <c r="I238" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="239" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="239" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A239">
         <v>1745</v>
       </c>
@@ -8717,10 +8735,10 @@
         <v>2958465</v>
       </c>
       <c r="I239" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="240" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="240" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A240">
         <v>1745</v>
       </c>
@@ -8746,10 +8764,10 @@
         <v>2958465</v>
       </c>
       <c r="I240" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="241" spans="1:9" x14ac:dyDescent="0.3">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="241" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A241">
         <v>1230</v>
       </c>
@@ -8775,10 +8793,10 @@
         <v>2958465</v>
       </c>
       <c r="I241" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="242" spans="1:9" x14ac:dyDescent="0.3">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="242" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A242">
         <v>2207</v>
       </c>
@@ -8804,10 +8822,10 @@
         <v>2958465</v>
       </c>
       <c r="I242" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="243" spans="1:9" x14ac:dyDescent="0.3">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="243" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A243">
         <v>2207</v>
       </c>
@@ -8833,10 +8851,10 @@
         <v>2958465</v>
       </c>
       <c r="I243" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="244" spans="1:9" x14ac:dyDescent="0.3">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="244" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A244">
         <v>2207</v>
       </c>
@@ -8862,10 +8880,10 @@
         <v>2958465</v>
       </c>
       <c r="I244" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="245" spans="1:9" x14ac:dyDescent="0.3">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="245" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A245">
         <v>2207</v>
       </c>
@@ -8891,10 +8909,10 @@
         <v>2958465</v>
       </c>
       <c r="I245" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="246" spans="1:9" x14ac:dyDescent="0.3">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="246" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A246">
         <v>2126</v>
       </c>
@@ -8920,10 +8938,10 @@
         <v>2958465</v>
       </c>
       <c r="I246" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="247" spans="1:9" x14ac:dyDescent="0.3">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="247" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A247">
         <v>2126</v>
       </c>
@@ -8949,10 +8967,10 @@
         <v>2958465</v>
       </c>
       <c r="I247" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="248" spans="1:9" x14ac:dyDescent="0.3">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="248" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A248">
         <v>2126</v>
       </c>
@@ -8978,10 +8996,10 @@
         <v>2958465</v>
       </c>
       <c r="I248" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="249" spans="1:9" x14ac:dyDescent="0.3">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="249" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A249">
         <v>2244</v>
       </c>
@@ -9007,10 +9025,10 @@
         <v>2958465</v>
       </c>
       <c r="I249" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="250" spans="1:9" x14ac:dyDescent="0.3">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="250" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A250">
         <v>2244</v>
       </c>
@@ -9036,10 +9054,10 @@
         <v>2958465</v>
       </c>
       <c r="I250" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="251" spans="1:9" x14ac:dyDescent="0.3">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="251" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A251">
         <v>2244</v>
       </c>
@@ -9065,10 +9083,10 @@
         <v>2958465</v>
       </c>
       <c r="I251" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="252" spans="1:9" x14ac:dyDescent="0.3">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="252" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A252">
         <v>2244</v>
       </c>
@@ -9094,10 +9112,10 @@
         <v>2958465</v>
       </c>
       <c r="I252" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="253" spans="1:9" x14ac:dyDescent="0.3">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="253" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A253">
         <v>2244</v>
       </c>
@@ -9123,10 +9141,10 @@
         <v>2958465</v>
       </c>
       <c r="I253" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="254" spans="1:9" x14ac:dyDescent="0.3">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="254" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A254">
         <v>1950</v>
       </c>
@@ -9152,10 +9170,10 @@
         <v>2958465</v>
       </c>
       <c r="I254" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="255" spans="1:9" x14ac:dyDescent="0.3">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="255" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A255">
         <v>1950</v>
       </c>
@@ -9181,10 +9199,10 @@
         <v>2958465</v>
       </c>
       <c r="I255" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="256" spans="1:9" x14ac:dyDescent="0.3">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="256" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A256">
         <v>2255</v>
       </c>
@@ -9210,10 +9228,10 @@
         <v>2958465</v>
       </c>
       <c r="I256" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="257" spans="1:9" x14ac:dyDescent="0.3">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="257" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257">
         <v>2250</v>
       </c>
@@ -9239,10 +9257,10 @@
         <v>2958465</v>
       </c>
       <c r="I257" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="258" spans="1:9" x14ac:dyDescent="0.3">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="258" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A258">
         <v>2250</v>
       </c>
@@ -9268,10 +9286,10 @@
         <v>2958465</v>
       </c>
       <c r="I258" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="259" spans="1:9" x14ac:dyDescent="0.3">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="259" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>2250</v>
       </c>
@@ -9297,10 +9315,10 @@
         <v>2958465</v>
       </c>
       <c r="I259" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="260" spans="1:9" x14ac:dyDescent="0.3">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="260" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A260">
         <v>2250</v>
       </c>
@@ -9326,10 +9344,10 @@
         <v>2958465</v>
       </c>
       <c r="I260" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="261" spans="1:9" x14ac:dyDescent="0.3">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="261" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A261">
         <v>2250</v>
       </c>
@@ -9355,10 +9373,10 @@
         <v>2958465</v>
       </c>
       <c r="I261" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="262" spans="1:9" x14ac:dyDescent="0.3">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="262" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A262">
         <v>2250</v>
       </c>
@@ -9384,10 +9402,17 @@
         <v>2958465</v>
       </c>
       <c r="I262" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I262" xr:uid="{9AECB136-8215-429B-82E5-8A6B6A669FFB}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="2258"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H262">
     <sortCondition ref="A2:A262"/>
     <sortCondition ref="B2:B262"/>
@@ -9399,12 +9424,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="MetaDocumentWS" ma:contentTypeID="0x01010002328573F07347D9A7800BDA19699CC200DE8F1DF1BF4211488DA32D5AC68DFB95" ma:contentTypeVersion="0" ma:contentTypeDescription="Metadata Content Type(Workshare)" ma:contentTypeScope="" ma:versionID="ea2efc4932be20cf5e8fe2ec0517f4d4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b6142cc285753f069fe6237cbe592e30">
     <xsd:element name="properties">
@@ -9518,16 +9552,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9975CE17-A2BF-4108-83DD-AD872CF67E1E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{034CDF24-425D-4892-AB7F-AACD3A1CB9F3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -9536,7 +9569,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D297E724-C9ED-40B8-8790-2B8BEFF24B33}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9550,12 +9583,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9975CE17-A2BF-4108-83DD-AD872CF67E1E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>